<commit_message>
Update Manage Taxes template to reflect recent changes in tax calculations
</commit_message>
<xml_diff>
--- a/Financials/Transaction Tax/Manage Taxes/Templates/Manage Taxes Tmpl.xlsx
+++ b/Financials/Transaction Tax/Manage Taxes/Templates/Manage Taxes Tmpl.xlsx
@@ -8,16 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Crist\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C72DD0-66BF-4BB9-9F6B-BA49030F191F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31414BA6-E655-491F-BDA1-F7428067F097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{6723E2BA-4745-4283-9749-DCFF573B2A3B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6723E2BA-4745-4283-9749-DCFF573B2A3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Doc" sheetId="3" r:id="rId1"/>
     <sheet name="Parmeters" sheetId="4" r:id="rId2"/>
     <sheet name="TaxRegime" sheetId="1" r:id="rId3"/>
-    <sheet name="Taxes" sheetId="5" r:id="rId4"/>
-    <sheet name="XDO_METADATA" sheetId="2" state="hidden" r:id="rId5"/>
+    <sheet name="Tax" sheetId="5" r:id="rId4"/>
+    <sheet name="DefaultTaxStatus" sheetId="6" r:id="rId5"/>
+    <sheet name="DefaultTaxRate" sheetId="9" r:id="rId6"/>
+    <sheet name="XDO_METADATA" sheetId="2" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="XDO_?XDOFIELD1?">Parmeters!$B$3</definedName>
@@ -32,30 +34,46 @@
     <definedName name="XDO_?XDOFIELD18?">TaxRegime!$Q$3</definedName>
     <definedName name="XDO_?XDOFIELD19?">Parmeters!$B$4</definedName>
     <definedName name="XDO_?XDOFIELD2?">TaxRegime!$A$3</definedName>
-    <definedName name="XDO_?XDOFIELD20?">Taxes!$A$3</definedName>
-    <definedName name="XDO_?XDOFIELD21?">Taxes!$B$3</definedName>
-    <definedName name="XDO_?XDOFIELD22?">Taxes!$C$3</definedName>
-    <definedName name="XDO_?XDOFIELD23?">Taxes!$D$3</definedName>
-    <definedName name="XDO_?XDOFIELD24?">Taxes!$E$3</definedName>
-    <definedName name="XDO_?XDOFIELD25?">Taxes!$F$3</definedName>
-    <definedName name="XDO_?XDOFIELD26?">Taxes!$G$3</definedName>
-    <definedName name="XDO_?XDOFIELD27?">Taxes!$H$3</definedName>
+    <definedName name="XDO_?XDOFIELD20?">Tax!$A$3</definedName>
+    <definedName name="XDO_?XDOFIELD21?">Tax!$B$3</definedName>
+    <definedName name="XDO_?XDOFIELD22?">Tax!$C$3</definedName>
+    <definedName name="XDO_?XDOFIELD23?">Tax!$D$3</definedName>
+    <definedName name="XDO_?XDOFIELD24?">Tax!$E$3</definedName>
+    <definedName name="XDO_?XDOFIELD25?">Tax!$F$3</definedName>
+    <definedName name="XDO_?XDOFIELD26?">Tax!$G$3</definedName>
+    <definedName name="XDO_?XDOFIELD27?">Tax!$H$3</definedName>
+    <definedName name="XDO_?XDOFIELD28?">DefaultTaxStatus!$A$3</definedName>
+    <definedName name="XDO_?XDOFIELD29?">DefaultTaxStatus!$B$3</definedName>
     <definedName name="XDO_?XDOFIELD3?">TaxRegime!$B$3</definedName>
+    <definedName name="XDO_?XDOFIELD30?">DefaultTaxStatus!$C$3</definedName>
+    <definedName name="XDO_?XDOFIELD31?">DefaultTaxStatus!$D$3</definedName>
+    <definedName name="XDO_?XDOFIELD32?">DefaultTaxStatus!$E$3</definedName>
+    <definedName name="XDO_?XDOFIELD33?">DefaultTaxStatus!$F$3</definedName>
+    <definedName name="XDO_?XDOFIELD34?">DefaultTaxRate!$A$3</definedName>
+    <definedName name="XDO_?XDOFIELD35?">DefaultTaxRate!$B$3</definedName>
+    <definedName name="XDO_?XDOFIELD36?">DefaultTaxRate!$C$3</definedName>
+    <definedName name="XDO_?XDOFIELD37?">DefaultTaxRate!$D$3</definedName>
+    <definedName name="XDO_?XDOFIELD38?">DefaultTaxRate!$E$3</definedName>
+    <definedName name="XDO_?XDOFIELD39?">DefaultTaxRate!$F$3</definedName>
     <definedName name="XDO_?XDOFIELD4?">TaxRegime!$C$3</definedName>
+    <definedName name="XDO_?XDOFIELD40?">DefaultTaxRate!$G$3</definedName>
+    <definedName name="XDO_?XDOFIELD41?">DefaultTaxRate!$H$3</definedName>
     <definedName name="XDO_?XDOFIELD5?">TaxRegime!$D$3</definedName>
     <definedName name="XDO_?XDOFIELD6?">TaxRegime!$E$3</definedName>
     <definedName name="XDO_?XDOFIELD7?">TaxRegime!$F$3</definedName>
     <definedName name="XDO_?XDOFIELD8?">TaxRegime!$G$3</definedName>
     <definedName name="XDO_?XDOFIELD9?">TaxRegime!$H$3</definedName>
     <definedName name="XDO_GROUP_?XDOG1?">TaxRegime!$A$3:$CA$3</definedName>
-    <definedName name="XDO_GROUP_?XDOG2?">Taxes!$A$3:$CA$3</definedName>
+    <definedName name="XDO_GROUP_?XDOG2?">Tax!$A$3:$CA$3</definedName>
+    <definedName name="XDO_GROUP_?XDOG3?">DefaultTaxStatus!$A$3:$CA$3</definedName>
+    <definedName name="XDO_GROUP_?XDOG4?">DefaultTaxRate!$A$3:$CA$3</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="160">
   <si>
     <t>Version</t>
   </si>
@@ -90,9 +108,6 @@
     <t>www.linkedin.com/in/cristian-arakaki</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/cristian-arakaki/</t>
-  </si>
-  <si>
     <t>26C</t>
   </si>
   <si>
@@ -138,139 +153,88 @@
     <t>XDO_?XDOFIELD2?</t>
   </si>
   <si>
-    <t>&lt;?TAX_REGIME_CODE?&gt;</t>
-  </si>
-  <si>
     <t>XDO_?XDOFIELD3?</t>
   </si>
   <si>
-    <t>&lt;?TAX_REGIME_NAME?&gt;</t>
-  </si>
-  <si>
     <t>AR</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD4?</t>
   </si>
   <si>
-    <t>&lt;?COUNTRY_CODE?&gt;</t>
-  </si>
-  <si>
     <t>1951-01-01T00:00:00.000+00:00</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD5?</t>
   </si>
   <si>
-    <t>&lt;?EFFECTIVE_FROM?&gt;</t>
-  </si>
-  <si>
     <t>EFFECTIVE_TO</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD6?</t>
   </si>
   <si>
-    <t>&lt;?EFFECTIVE_TO?&gt;</t>
-  </si>
-  <si>
     <t>ARS</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD7?</t>
   </si>
   <si>
-    <t>&lt;?TAX_CURRENCY_CODE?&gt;</t>
-  </si>
-  <si>
     <t>XDO_?XDOFIELD8?</t>
   </si>
   <si>
-    <t>&lt;?MINIMUM_ACCOUNTABLE_UNIT?&gt;</t>
-  </si>
-  <si>
     <t>XDO_?XDOFIELD9?</t>
   </si>
   <si>
-    <t>&lt;?TAX_PRECISION?&gt;</t>
-  </si>
-  <si>
     <t>NEAREST</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD10?</t>
   </si>
   <si>
-    <t>&lt;?ROUNDING_RULE_CODE?&gt;</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD11?</t>
   </si>
   <si>
-    <t>&lt;?ALLOW_ROUNDING_OVERRIDE_FLAG?&gt;</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD12?</t>
   </si>
   <si>
-    <t>&lt;?REGN_NUM_SAME_AS_LE_FLAG?&gt;</t>
-  </si>
-  <si>
     <t>L</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD13?</t>
   </si>
   <si>
-    <t>&lt;?BUCKET_LEVEL_FLAG?&gt;</t>
-  </si>
-  <si>
     <t>VALIDATION_TYPE</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD14?</t>
   </si>
   <si>
-    <t>&lt;?VALIDATION_TYPE?&gt;</t>
-  </si>
-  <si>
     <t>VALIDATION_LEVEL</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD15?</t>
   </si>
   <si>
-    <t>&lt;?VALIDATION_LEVEL?&gt;</t>
-  </si>
-  <si>
     <t>UNIQUENESS_VALIDATION_LEVEL</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD16?</t>
   </si>
   <si>
-    <t>&lt;?UNIQUENESS_VALIDATION_LEVEL?&gt;</t>
-  </si>
-  <si>
     <t>XDO_?XDOFIELD17?</t>
   </si>
   <si>
-    <t>&lt;?CROSS_REGIME_COMPOUNDING_FLAG?&gt;</t>
-  </si>
-  <si>
     <t>REGIME_PRECEDENCE</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD18?</t>
-  </si>
-  <si>
-    <t>&lt;?REGIME_PRECEDENCE?&gt;</t>
   </si>
   <si>
     <t>Tax Regime Code</t>
@@ -367,24 +331,15 @@
     <t>XDO_?XDOFIELD21?</t>
   </si>
   <si>
-    <t>&lt;?CONTENT_OWNER_ID?&gt;</t>
-  </si>
-  <si>
     <t>RET GAN HONORARIOS PROF RI</t>
   </si>
   <si>
     <t>XDO_?XDOFIELD22?</t>
   </si>
   <si>
-    <t>&lt;?TAX?&gt;</t>
-  </si>
-  <si>
     <t>XDO_?XDOFIELD23?</t>
   </si>
   <si>
-    <t>&lt;?TAX_FULL_NAME?&gt;</t>
-  </si>
-  <si>
     <t>XDO_?XDOFIELD24?</t>
   </si>
   <si>
@@ -394,15 +349,9 @@
     <t>XDO_?XDOFIELD26?</t>
   </si>
   <si>
-    <t>&lt;?ALLOW_EXCEPTIONS_FLAG?&gt;</t>
-  </si>
-  <si>
     <t>XDO_?XDOFIELD27?</t>
   </si>
   <si>
-    <t>&lt;?ALLOW_EXEMPTIONS_FLAG?&gt;</t>
-  </si>
-  <si>
     <t>Configuration Owner</t>
   </si>
   <si>
@@ -425,6 +374,186 @@
   </si>
   <si>
     <t>&lt;xsl:for-each select=".//G_2"&gt;</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD28?</t>
+  </si>
+  <si>
+    <t>RET GAN HONORARIOS RNI EST</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>RET GAN HONORARIOS RNI</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD29?</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD30?</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD31?</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD32?</t>
+  </si>
+  <si>
+    <t>DEFAULT_FLG_EFFECTIVE_TO</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD33?</t>
+  </si>
+  <si>
+    <t>Default flag</t>
+  </si>
+  <si>
+    <t>Default Start Date</t>
+  </si>
+  <si>
+    <t>Default End Date</t>
+  </si>
+  <si>
+    <t>XDO_GROUP_?XDOG3?</t>
+  </si>
+  <si>
+    <t>&lt;xsl:for-each select=".//G_3"&gt;</t>
+  </si>
+  <si>
+    <t>Rate</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD34?</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD35?</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD36?</t>
+  </si>
+  <si>
+    <t>GAN HONORARIOS RNI</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD37?</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD38?</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD39?</t>
+  </si>
+  <si>
+    <t>2023-09-30T00:00:00.000+00:00</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD40?</t>
+  </si>
+  <si>
+    <t>Tax Rate Type</t>
+  </si>
+  <si>
+    <t>PERCENTAGE</t>
+  </si>
+  <si>
+    <t>XDO_?XDOFIELD41?</t>
+  </si>
+  <si>
+    <t>XDO_GROUP_?XDOG4?</t>
+  </si>
+  <si>
+    <t>&lt;xsl:for-each select=".//G_4"&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./COUNTRY_CODE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX_REGIME_CODE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX_REGIME_NAME?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./EFFECTIVE_FROM?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./EFFECTIVE_TO?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX_CURRENCY_CODE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./MINIMUM_ACCOUNTABLE_UNIT?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX_PRECISION?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./ROUNDING_RULE_CODE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./ALLOW_ROUNDING_OVERRIDE_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./REGN_NUM_SAME_AS_LE_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./BUCKET_LEVEL_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./VALIDATION_TYPE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./VALIDATION_LEVEL?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./UNIQUENESS_VALIDATION_LEVEL?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./CROSS_REGIME_COMPOUNDING_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./REGIME_PRECEDENCE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./CONTENT_OWNER_ID?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX_FULL_NAME?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./ALLOW_EXCEPTIONS_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./ALLOW_EXEMPTIONS_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX_STATUS_CODE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./DEFAULT_STATUS_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./DEFAULT_FLG_EFFECTIVE_FROM?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./DEFAULT_FLG_EFFECTIVE_TO?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./TAX_RATE_CODE?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./DEFAULT_RATE_FLAG?&gt;</t>
+  </si>
+  <si>
+    <t>&lt;?./RATE_TYPE_CODE?&gt;</t>
+  </si>
+  <si>
+    <t>https://github.com/carakaki</t>
   </si>
 </sst>
 </file>
@@ -876,50 +1005,50 @@
   <sheetData>
     <row r="2" spans="1:2">
       <c r="A2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30">
       <c r="A3" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>17</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>11</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" s="13">
-        <v>46314</v>
+        <v>46320</v>
       </c>
     </row>
   </sheetData>
@@ -941,23 +1070,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="10" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -977,86 +1106,86 @@
   <sheetData>
     <row r="1" spans="1:17">
       <c r="G1" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="M1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="P1" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" s="10" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:17">
       <c r="A3" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>33</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>39</v>
       </c>
       <c r="G3" s="11">
         <v>0.01</v>
@@ -1065,31 +1194,31 @@
         <v>2</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="J3" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="O3" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="P3" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q3" s="11" t="s">
         <v>52</v>
-      </c>
-      <c r="L3" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="M3" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="N3" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="P3" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1106,59 +1235,59 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="G1" t="s">
-        <v>118</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="10" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>115</v>
+        <v>92</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11">
         <v>-99</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1167,8 +1296,123 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853B4E0C-D2C5-4BB1-93A8-398D0DE63BAC}">
+  <dimension ref="A2:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6">
+      <c r="A2" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D69CE90-7AA4-48F9-A1B6-36DE16A9F06C}">
+  <dimension ref="A2:H3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2" spans="1:8">
+      <c r="A2" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14B3D414-768A-4269-855B-4335A4220462}">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
@@ -1181,7 +1425,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1">
@@ -1195,7 +1439,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1223,7 +1467,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="8">
-        <v>46314</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1242,240 +1486,374 @@
     </row>
     <row r="11" spans="1:2" s="5" customFormat="1" ht="14.25">
       <c r="A11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="5" customFormat="1" ht="14.25">
       <c r="A12" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>27</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="5" customFormat="1" ht="14.25">
       <c r="A13" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="5" customFormat="1" ht="14.25">
       <c r="A14" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>32</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="5" customFormat="1" ht="14.25">
       <c r="A15" s="5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>35</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:2" s="5" customFormat="1" ht="14.25">
       <c r="A16" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>38</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:3" s="5" customFormat="1" ht="14.25">
       <c r="A17" s="5" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>41</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:3" s="5" customFormat="1" ht="14.25">
       <c r="A18" s="5" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>43</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:3" s="5" customFormat="1" ht="14.25">
       <c r="A19" s="5" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>45</v>
+        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B22" t="s">
-        <v>54</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>63</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B26" t="s">
-        <v>66</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>68</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>71</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="B30" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="B31" t="s">
-        <v>27</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="B32" t="s">
-        <v>103</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="B33" t="s">
-        <v>106</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="B34" t="s">
-        <v>108</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="B37" t="s">
-        <v>112</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="B38" t="s">
-        <v>114</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>100</v>
+      </c>
+      <c r="B40" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>105</v>
+      </c>
+      <c r="B42" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>107</v>
+      </c>
+      <c r="B44" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>109</v>
+      </c>
+      <c r="B45" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>113</v>
+      </c>
+      <c r="B46" t="s">
+        <v>114</v>
+      </c>
+      <c r="C46" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>116</v>
+      </c>
+      <c r="B47" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>117</v>
+      </c>
+      <c r="B48" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>118</v>
+      </c>
+      <c r="B49" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>120</v>
+      </c>
+      <c r="B50" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
         <v>121</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
         <v>122</v>
       </c>
-      <c r="C39" t="s">
-        <v>94</v>
+      <c r="B52" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>124</v>
+      </c>
+      <c r="B53" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>127</v>
+      </c>
+      <c r="B54" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>128</v>
+      </c>
+      <c r="B55" t="s">
+        <v>129</v>
+      </c>
+      <c r="C55" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1484,6 +1862,6 @@
     <hyperlink ref="B8" r:id="rId1" xr:uid="{2A15A0EF-6E40-47B3-91C6-E1C0F2007E1E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>